<commit_message>
Fix digestate math and goat seasonality in coefficient examples
The Example Results sheet computed monthly digestate as (daily dung x
1.5) without multiplying by 30 days, understating fertilizer value and
total savings by 30x. Also updated the goat example to match the app's
year-round calculation instead of the old April-October only model.
</commit_message>
<xml_diff>
--- a/docs/biogas-coefficients.xlsx
+++ b/docs/biogas-coefficients.xlsx
@@ -315,6 +315,12 @@
   </si>
   <si>
     <t xml:space="preserve">GOAT </t>
+  </si>
+  <si>
+    <t>EXAMPLE 3: ONE GOAT</t>
+  </si>
+  <si>
+    <t>PKR/year from 1 goat</t>
   </si>
 </sst>
 </file>
@@ -1123,7 +1129,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:C35"/>
+  <dimension ref="A1:C37"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="35" customWidth="1"/>
@@ -1214,7 +1220,7 @@
         <v>61</v>
       </c>
       <c r="B10" s="8">
-        <v>22.5</v>
+        <v>675</v>
       </c>
       <c r="C10" t="s">
         <v>62</v>
@@ -1225,7 +1231,7 @@
         <v>63</v>
       </c>
       <c r="B11" s="9">
-        <v>337</v>
+        <v>10125</v>
       </c>
       <c r="C11" t="s">
         <v>58</v>
@@ -1236,7 +1242,7 @@
         <v>64</v>
       </c>
       <c r="B12" s="9">
-        <v>4044</v>
+        <v>121500</v>
       </c>
       <c r="C12" t="s">
         <v>60</v>
@@ -1247,7 +1253,7 @@
         <v>65</v>
       </c>
       <c r="B13" s="9">
-        <v>21744</v>
+        <v>139200</v>
       </c>
       <c r="C13" t="s">
         <v>66</v>
@@ -1334,7 +1340,7 @@
         <v>61</v>
       </c>
       <c r="B22" s="8">
-        <v>14.25</v>
+        <v>427.5</v>
       </c>
       <c r="C22" t="s">
         <v>62</v>
@@ -1345,7 +1351,7 @@
         <v>63</v>
       </c>
       <c r="B23" s="9">
-        <v>214</v>
+        <v>6413</v>
       </c>
       <c r="C23" t="s">
         <v>58</v>
@@ -1356,7 +1362,7 @@
         <v>64</v>
       </c>
       <c r="B24" s="9">
-        <v>2568</v>
+        <v>76950</v>
       </c>
       <c r="C24" t="s">
         <v>60</v>
@@ -1367,7 +1373,7 @@
         <v>65</v>
       </c>
       <c r="B25" s="9">
-        <v>36468</v>
+        <v>110850</v>
       </c>
       <c r="C25" t="s">
         <v>68</v>
@@ -1378,7 +1384,7 @@
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" s="14" t="s">
-        <v>69</v>
+        <v>93</v>
       </c>
       <c r="B27" s="15"/>
       <c r="C27" s="12"/>
@@ -1396,7 +1402,7 @@
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>70</v>
+        <v>51</v>
       </c>
       <c r="B29" s="8">
         <v>0.61</v>
@@ -1407,10 +1413,10 @@
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>71</v>
+        <v>53</v>
       </c>
       <c r="B30" s="8">
-        <v>18.399999999999999</v>
+        <v>18.4</v>
       </c>
       <c r="C30" t="s">
         <v>54</v>
@@ -1421,7 +1427,7 @@
         <v>55</v>
       </c>
       <c r="B31" s="8">
-        <v>9.6999999999999993</v>
+        <v>9.7</v>
       </c>
       <c r="C31" t="s">
         <v>56</v>
@@ -1435,38 +1441,62 @@
         <v>2425</v>
       </c>
       <c r="C32" t="s">
-        <v>72</v>
+        <v>58</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>73</v>
+        <v>59</v>
       </c>
       <c r="B33" s="9">
-        <v>16975</v>
+        <v>29100</v>
       </c>
       <c r="C33" t="s">
-        <v>74</v>
+        <v>60</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>75</v>
-      </c>
-      <c r="B34" s="9">
-        <v>14143</v>
+        <v>61</v>
+      </c>
+      <c r="B34" s="8">
+        <v>78.75</v>
       </c>
       <c r="C34" t="s">
-        <v>76</v>
+        <v>62</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>77</v>
-      </c>
-      <c r="B35" s="8"/>
+        <v>63</v>
+      </c>
+      <c r="B35" s="9">
+        <v>1181</v>
+      </c>
       <c r="C35" t="s">
-        <v>78</v>
+        <v>58</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>64</v>
+      </c>
+      <c r="B36" s="9">
+        <v>14175</v>
+      </c>
+      <c r="C36" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>65</v>
+      </c>
+      <c r="B37" s="9">
+        <v>43275</v>
+      </c>
+      <c r="C37" t="s">
+        <v>94</v>
       </c>
     </row>
   </sheetData>

</xml_diff>